<commit_message>
Cleanup and make radius unique
</commit_message>
<xml_diff>
--- a/test_locations.xlsx
+++ b/test_locations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,11 @@
           <t>longitude</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>radius</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -434,6 +439,9 @@
       </c>
       <c r="B2" t="n">
         <v>-74.006</v>
+      </c>
+      <c r="C2" t="n">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>